<commit_message>
Per-person weekly off: admin sets it per staff (table, profile form, Excel import); attendance, absents, leave balance, payroll and Simran use it
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/templates/staff-import-template.xlsx
+++ b/public/templates/staff-import-template.xlsx
@@ -113,12 +113,20 @@
         </r>
       </text>
     </comment>
+    <comment ref="M1" authorId="0">
+      <text>
+        <r>
+          <t xml:space="preserve">Weekly off
+Sunday (default) · Saturday · "Sat, Sun" etc.</t>
+        </r>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="68">
   <si>
     <t>name</t>
   </si>
@@ -156,6 +164,9 @@
     <t>reporting_manager</t>
   </si>
   <si>
+    <t>week_off</t>
+  </si>
+  <si>
     <t>Giriraj Sahu</t>
   </si>
   <si>
@@ -216,6 +227,9 @@
     <t>1995-01-30</t>
   </si>
   <si>
+    <t>Saturday</t>
+  </si>
+  <si>
     <t>Arjun Khanna</t>
   </si>
   <si>
@@ -237,6 +251,9 @@
     <t>2000-12-05</t>
   </si>
   <si>
+    <t>Sat, Sun</t>
+  </si>
+  <si>
     <t>Lighthouse · Staff import</t>
   </si>
   <si>
@@ -292,6 +309,9 @@
   </si>
   <si>
     <t>Reporting manager — Name of the manager, optional</t>
+  </si>
+  <si>
+    <t>Weekly off — Sunday (default) · Saturday · "Sat, Sun" etc.</t>
   </si>
   <si>
     <t>Rules</t>
@@ -736,7 +756,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L60"/>
+  <dimension ref="A1:M60"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -748,9 +768,10 @@
     <col min="9" max="9" width="18" customWidth="1"/>
     <col min="10" max="11" width="14" customWidth="1"/>
     <col min="12" max="12" width="22" customWidth="1"/>
+    <col min="13" max="13" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="20" customHeight="1" spans="1:12" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" ht="20" customHeight="1" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -787,119 +808,131 @@
       <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="2" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="I2" s="3">
         <v>42000</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="L2" s="2" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+      <c r="M2" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="I3" s="3">
         <v>32000</v>
       </c>
       <c r="J3" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="K3" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="L3" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="M3" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="H4" s="2" t="s">
         <v>30</v>
-      </c>
-      <c r="K3" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="L3" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="H4" s="2" t="s">
-        <v>29</v>
       </c>
       <c r="I4" s="3">
         <v>30000</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="L4" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="M4" s="2" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="5" spans="9:9" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -1090,7 +1123,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B25"/>
+  <dimension ref="A1:B26"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -1099,58 +1132,58 @@
   <sheetData>
     <row r="1" spans="1:2" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="2" spans="1:2" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="3" spans="1:2" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
     </row>
     <row r="4" spans="1:2" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="5" spans="1:2" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
     </row>
     <row r="6" spans="1:2" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="7" spans="1:2" s="9" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="9" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
     </row>
     <row r="8" spans="1:2" s="7" customFormat="1" x14ac:dyDescent="0.25">
@@ -1158,7 +1191,7 @@
         <v>0</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
     </row>
     <row r="9" spans="1:2" s="7" customFormat="1" x14ac:dyDescent="0.25">
@@ -1166,7 +1199,7 @@
         <v>1</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
     </row>
     <row r="10" spans="1:2" s="7" customFormat="1" x14ac:dyDescent="0.25">
@@ -1174,7 +1207,7 @@
         <v>2</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
     </row>
     <row r="11" spans="1:2" s="7" customFormat="1" x14ac:dyDescent="0.25">
@@ -1182,7 +1215,7 @@
         <v>3</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
     </row>
     <row r="12" spans="1:2" s="7" customFormat="1" x14ac:dyDescent="0.25">
@@ -1190,7 +1223,7 @@
         <v>4</v>
       </c>
       <c r="B12" s="7" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
     </row>
     <row r="13" spans="1:2" s="7" customFormat="1" x14ac:dyDescent="0.25">
@@ -1198,7 +1231,7 @@
         <v>5</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
     </row>
     <row r="14" spans="1:2" s="7" customFormat="1" x14ac:dyDescent="0.25">
@@ -1206,7 +1239,7 @@
         <v>6</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
     </row>
     <row r="15" spans="1:2" s="7" customFormat="1" x14ac:dyDescent="0.25">
@@ -1214,7 +1247,7 @@
         <v>7</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
     </row>
     <row r="16" spans="1:2" s="7" customFormat="1" x14ac:dyDescent="0.25">
@@ -1222,7 +1255,7 @@
         <v>8</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
     </row>
     <row r="17" spans="1:2" s="7" customFormat="1" x14ac:dyDescent="0.25">
@@ -1230,7 +1263,7 @@
         <v>9</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
     </row>
     <row r="18" spans="1:2" s="7" customFormat="1" x14ac:dyDescent="0.25">
@@ -1238,7 +1271,7 @@
         <v>10</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
     </row>
     <row r="19" spans="1:2" s="7" customFormat="1" x14ac:dyDescent="0.25">
@@ -1246,55 +1279,63 @@
         <v>11</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
     </row>
     <row r="20" spans="1:2" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="7" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>14</v>
+        <v>61</v>
       </c>
     </row>
     <row r="21" spans="1:2" s="7" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="8" t="s">
-        <v>58</v>
+      <c r="A21" s="7" t="s">
+        <v>15</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>59</v>
+        <v>15</v>
       </c>
     </row>
     <row r="22" spans="1:2" s="7" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="7" t="s">
-        <v>14</v>
+      <c r="A22" s="8" t="s">
+        <v>62</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
     </row>
     <row r="23" spans="1:2" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="7" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
     </row>
     <row r="24" spans="1:2" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="7" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
     </row>
     <row r="25" spans="1:2" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="7" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B25" s="7" t="s">
-        <v>63</v>
+        <v>66</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="B26" s="7" t="s">
+        <v>67</v>
       </c>
     </row>
   </sheetData>

</xml_diff>